<commit_message>
Simplificar: solo 2 Excel (Anexo_validado + Anexo_limpio) y 2 validaciones
- Anexo_validado.xlsx: datos originales del Anexo1 SIN correcciones
  + Validacion_1: Completo / Incompleto / Error (detalla que campo)
  + Validacion_2: diferencias con Vinculaciones y Base Inversiones
  + Hojas: Diccionario de Datos, Diccionario de Errores

- Anexo_limpio.xlsx: CON correcciones de bases maestras aplicadas
  + Recalcula Validacion_1 despues de aplicar correcciones

- Eliminados: Anexo1_base_limpia, Anexo1_base_errores, Anexo1_base_excluidos
- Eliminados: campos err_* individuales, status, campos_faltantes

https://claude.ai/code/session_0121JkH5k2aVGJTB7hSBSGGB
</commit_message>
<xml_diff>
--- a/Anexo1_reporte.xlsx
+++ b/Anexo1_reporte.xlsx
@@ -446,17 +446,17 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>LIMPIO</t>
+          <t>Completo</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>CON ERRORES</t>
+          <t>Incompleto</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>EXCLUIDO</t>
+          <t>Con Error</t>
         </is>
       </c>
     </row>
@@ -510,10 +510,10 @@
         <v>164</v>
       </c>
       <c r="G3" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="H3" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -538,10 +538,10 @@
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H4" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
@@ -594,10 +594,10 @@
         <v>40</v>
       </c>
       <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
         <v>7</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -622,10 +622,10 @@
         <v>10</v>
       </c>
       <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>5</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -650,10 +650,10 @@
         <v>7</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9">
@@ -678,10 +678,10 @@
         <v>71</v>
       </c>
       <c r="G9" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="H9" t="n">
-        <v>16</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
@@ -706,10 +706,10 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -734,10 +734,10 @@
         <v>5</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H11" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -790,10 +790,10 @@
         <v>37</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H13" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -902,10 +902,10 @@
         <v>5</v>
       </c>
       <c r="G17" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" t="n">
         <v>1</v>
-      </c>
-      <c r="H17" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -930,10 +930,10 @@
         <v>4</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -986,10 +986,10 @@
         <v>41</v>
       </c>
       <c r="G20" t="n">
+        <v>13</v>
+      </c>
+      <c r="H20" t="n">
         <v>3</v>
-      </c>
-      <c r="H20" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="21">
@@ -1014,10 +1014,10 @@
         <v>3</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="H21" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1042,10 +1042,10 @@
         <v>40</v>
       </c>
       <c r="G22" t="n">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="H22" t="n">
-        <v>52</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23">
@@ -1098,10 +1098,10 @@
         <v>5</v>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="H24" t="n">
-        <v>69</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25">
@@ -1126,10 +1126,10 @@
         <v>3</v>
       </c>
       <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
         <v>3</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1154,10 +1154,10 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" t="n">
         <v>5</v>
-      </c>
-      <c r="H26" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="27">
@@ -1182,10 +1182,10 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1210,10 +1210,10 @@
         <v>431</v>
       </c>
       <c r="G28" t="n">
-        <v>2</v>
+        <v>75</v>
       </c>
       <c r="H28" t="n">
-        <v>77</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1227,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>cantidad_errores</t>
+          <t>cantidad</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -1269,7 +1269,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5">
@@ -1279,117 +1279,127 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>57</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>comp</t>
+          <t>f9</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>unid</t>
+          <t>comp</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>55</v>
+        <v>354</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>demol</t>
+          <t>unid</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>nueva</t>
+          <t>demol</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>reforz</t>
+          <t>nueva</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cerco</t>
+          <t>reforz</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>17</v>
+        <v>142</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>sust</t>
+          <t>cerco</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>16</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ampl</t>
+          <t>sust</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>17</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>mobil</t>
+          <t>ampl</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>17</v>
+        <v>146</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>agua</t>
+          <t>mobil</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>17</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>agua</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>elec</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>26</v>
+      <c r="B17" t="n">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -1403,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1455,7 +1465,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Registros limpios</t>
+          <t>Completos</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1465,21 +1475,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Registros con errores</t>
+          <t>Incompletos</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>78</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Registros excluidos</t>
+          <t>Con errores</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>375</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9">
@@ -1489,10 +1499,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Correcciones realizadas</t>
+          <t>Con diferencias vs maestras</t>
         </is>
       </c>
       <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Correcciones en Anexo_limpio</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>